<commit_message>
Make demo account names generic
</commit_message>
<xml_diff>
--- a/整理后数据/2501/信用卡9001_2501.xlsx
+++ b/整理后数据/2501/信用卡9001_2501.xlsx
@@ -515,7 +515,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>示例银行A信用卡9001</t>
+          <t>示例银行A信用卡</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -528,7 +528,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>示例银行A信用卡9001</t>
+          <t>示例银行A信用卡</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>示例银行A信用卡9001</t>
+          <t>示例银行A信用卡</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -577,7 +577,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>示例银行A信用卡9001</t>
+          <t>示例银行A信用卡</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>示例银行A信用卡9001</t>
+          <t>示例银行A信用卡</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -626,7 +626,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>示例银行A信用卡9001</t>
+          <t>示例银行A信用卡</t>
         </is>
       </c>
     </row>

</xml_diff>